<commit_message>
update uploader to target sheet name
</commit_message>
<xml_diff>
--- a/public/uploaders/ADVISORY-CLASS-UPLOADER-SHS-NEW.xlsx
+++ b/public/uploaders/ADVISORY-CLASS-UPLOADER-SHS-NEW.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RBIS07\Desktop\Systems\System Files\STARS\Uploader\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\var\www\laravel\stars\public\uploaders\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18D1613B-17B9-43F2-A563-5F54E565DE8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{661EC825-6421-49F6-8E00-1F7C3F08E051}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="REFERENCE " sheetId="2" state="hidden" r:id="rId1"/>
     <sheet name="Instruction" sheetId="8" r:id="rId2"/>
-    <sheet name="Encode Here" sheetId="7" r:id="rId3"/>
+    <sheet name="ENCODE here" sheetId="7" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Encode Here'!$J$3:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ENCODE here'!$J$3:$J$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Instruction!$J$3:$J$6</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -917,14 +917,14 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2804,8 +2804,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="14014938" y="5279292"/>
-          <a:ext cx="0" cy="3898218"/>
+          <a:off x="14020800" y="5297714"/>
+          <a:ext cx="0" cy="3909941"/>
           <a:chOff x="13344072" y="5632530"/>
           <a:chExt cx="6542940" cy="4964868"/>
         </a:xfrm>
@@ -2988,73 +2988,73 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table225" displayName="Table225" ref="J2:J6" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table225" displayName="Table225" ref="J2:J6" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
   <autoFilter ref="J2:J6" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Academic " dataDxfId="37"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Academic " dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table446" displayName="Table446" ref="K2:W57" totalsRowShown="0" headerRowDxfId="36" dataDxfId="34" headerRowBorderDxfId="35" tableBorderDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table446" displayName="Table446" ref="K2:W57" totalsRowShown="0" headerRowDxfId="16" dataDxfId="14" headerRowBorderDxfId="15" tableBorderDxfId="13">
   <autoFilter ref="K2:W57" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Technical-Vocational-Livelihood " dataDxfId="32"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Sports " dataDxfId="31"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Arts and Design Track" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Accountancy, Business and Management Strand (ABM)" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Humanities and Social Sciences Strand (HUMMS)" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Science, Technology, Engineering and Mathematics Strand (STEM)" dataDxfId="27"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="General Academic Strand" dataDxfId="26"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Agri-Fishery Arts" dataDxfId="25"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Home Economics" dataDxfId="24"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="Industrial Arts" dataDxfId="23"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Information and Communication Technology (ICT)" dataDxfId="22"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Sports" dataDxfId="21"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Arts &amp; Design" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Technical-Vocational-Livelihood " dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Sports " dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Arts and Design Track" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Accountancy, Business and Management Strand (ABM)" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Humanities and Social Sciences Strand (HUMMS)" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Science, Technology, Engineering and Mathematics Strand (STEM)" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="General Academic Strand" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Agri-Fishery Arts" dataDxfId="5"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Home Economics" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="Industrial Arts" dataDxfId="3"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Information and Communication Technology (ICT)" dataDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Sports" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Arts &amp; Design" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table22" displayName="Table22" ref="J2:J6" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table22" displayName="Table22" ref="J2:J6" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
   <autoFilter ref="J2:J6" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Academic " dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Academic " dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table44" displayName="Table44" ref="K2:W57" totalsRowShown="0" headerRowDxfId="16" dataDxfId="14" headerRowBorderDxfId="15" tableBorderDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table44" displayName="Table44" ref="K2:W57" totalsRowShown="0" headerRowDxfId="36" dataDxfId="34" headerRowBorderDxfId="35" tableBorderDxfId="33">
   <autoFilter ref="K2:W57" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Technical-Vocational-Livelihood " dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Sports " dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Arts and Design Track" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Accountancy, Business and Management Strand (ABM)" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Humanities and Social Sciences Strand (HUMMS)" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Science, Technology, Engineering and Mathematics Strand (STEM)" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="General Academic Strand" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="Agri-Fishery Arts" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="Home Economics" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="Industrial Arts" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="Information and Communication Technology (ICT)" dataDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0300-00000C000000}" name="Sports" dataDxfId="1"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0300-00000D000000}" name="Arts &amp; Design" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Technical-Vocational-Livelihood " dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Sports " dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Arts and Design Track" dataDxfId="30"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Accountancy, Business and Management Strand (ABM)" dataDxfId="29"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Humanities and Social Sciences Strand (HUMMS)" dataDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Science, Technology, Engineering and Mathematics Strand (STEM)" dataDxfId="27"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="General Academic Strand" dataDxfId="26"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="Agri-Fishery Arts" dataDxfId="25"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="Home Economics" dataDxfId="24"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="Industrial Arts" dataDxfId="23"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="Information and Communication Technology (ICT)" dataDxfId="22"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0300-00000C000000}" name="Sports" dataDxfId="21"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0300-00000D000000}" name="Arts &amp; Design" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3092,7 +3092,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3198,7 +3198,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3340,7 +3340,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3363,33 +3363,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
       <c r="G1" s="5"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25" t="s">
+      <c r="B2" s="26"/>
+      <c r="C2" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25" t="s">
+      <c r="D2" s="26"/>
+      <c r="E2" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25" t="s">
+      <c r="F2" s="26"/>
+      <c r="G2" s="26" t="s">
         <v>180</v>
       </c>
-      <c r="H2" s="25"/>
+      <c r="H2" s="26"/>
       <c r="I2" s="12" t="s">
         <v>198</v>
       </c>
@@ -3664,7 +3664,7 @@
       <c r="C25" s="9">
         <v>1.3</v>
       </c>
-      <c r="D25" s="26" t="s">
+      <c r="D25" s="27" t="s">
         <v>12</v>
       </c>
       <c r="F25" s="6" t="s">
@@ -3673,7 +3673,7 @@
     </row>
     <row r="26" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C26" s="9"/>
-      <c r="D26" s="26"/>
+      <c r="D26" s="27"/>
       <c r="F26" s="6" t="s">
         <v>32</v>
       </c>
@@ -4445,15 +4445,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
     </row>
     <row r="2" spans="1:23" s="13" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -7318,15 +7318,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
     </row>
     <row r="2" spans="1:23" s="13" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">

</xml_diff>